<commit_message>
fix: add alias of some courses
Signed-off-by: Fovir <fovir@disroot.org>
</commit_message>
<xml_diff>
--- a/data/training-list.xlsx
+++ b/data/training-list.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="82">
   <si>
     <t xml:space="preserve">Training</t>
   </si>
@@ -31,194 +31,242 @@
     <t xml:space="preserve">No of Hours (Training)</t>
   </si>
   <si>
+    <t xml:space="preserve">Career in Cybersecurity - Entry Level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 Hours​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Career Paths in Cybersecurity​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Careers in Cybersecurity: Entry​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Careers in Cybersecurity: Expert​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intermediate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Careers in Cybersecurity: Management​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advanced</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Careers in Cybersecurity: Specialist​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cloud Architecture &amp; Security in AWS </t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CompTIA A+​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 Days​ (40 hours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CompTIA Cybersecurity Analyst (CySA+)​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CompTIA CySA+ Certification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CompTIA Linux+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CompTIA Network+ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CompTIA Network+ Certification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CompTIA PenTest+​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CompTIA PenTest+ Certification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CompTIA Security+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CompTIA Security+ Certification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CompTIA ​Server+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CompTIA Server+ Certification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CompTIA Tech+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 Days​ (24 hours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cybersecurity &amp; AI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 Hours</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cybersecurity Awareness</t>
   </si>
   <si>
-    <t xml:space="preserve">Entry</t>
-  </si>
-  <si>
     <t xml:space="preserve">3 Hours​</t>
   </si>
   <si>
+    <t xml:space="preserve">Cybersecurity Tools</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EC-Council  Certified Ethical Hacker (CEH)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EC-Council Certified Chief Information Security Officer (CCISO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identity &amp; Access Management (IAM) (Intermediate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 days (12 hours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identity &amp; Access Management (IAM) Intermediate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incident Response, Threat Intelligence &amp; Digital Forensic Investigators </t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 Days​ (35 hours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Information Technology - Computer Essentials​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 day (6 hours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Information Technology - Networking Essentials​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Information Technology - Security Essentials​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Introduction to Cloud Computing​</t>
+  </si>
+  <si>
     <t xml:space="preserve">Introduction to Cybersecurity​</t>
   </si>
   <si>
-    <t xml:space="preserve">2 days (12 hours)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Information Technology - Computer Essentials​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 day (6 hours)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Information Technology - Networking Essentials​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Information Technology - Security Essentials​</t>
+    <t xml:space="preserve">Introduction to Identity &amp; Access Management (IAM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 Hours​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Introduction to Identity &amp; Access Management (IAM) ​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Introduction to Mobile Security</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Introduction to Mobile Security Technology​</t>
   </si>
   <si>
     <t xml:space="preserve">Introduction to Python</t>
   </si>
   <si>
-    <t xml:space="preserve">Introduction to Cloud Computing​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 Hours​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Introduction to Mobile Security Technology​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Introduction to Identity &amp; Access Management (IAM) ​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 Hours​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cybersecurity Tools</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Intermediate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 Hours</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cybersecurity &amp; AI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scripting for Cybersecurity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reverse Malware Engineering</t>
+    <t xml:space="preserve">ISC2 Certified in Cybersecurity </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISC2 Certified in Cybersecurity Certification (CC)​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISC2 Certified Information Systems Security Professional (CISSP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISC2 Certified Information Systems Security Professional Certification (CISSP)​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISC2 Certified Secure Software Lifecycle Professional (CSSLP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISC2 Governance, Risk and Compliance Certification (CGRC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISC2 Systems Security Certified Practitioner (SSCP)</t>
   </si>
   <si>
     <t xml:space="preserve">Mobile Security 
 Intermediate</t>
   </si>
   <si>
-    <t xml:space="preserve">Identity &amp; Access Management (IAM) Intermediate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cloud Architecture &amp; Security in AWS </t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 days</t>
+    <t xml:space="preserve">Mobile Security (Intermediate)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PECB Certified Chief ​Information Security Officer (CISO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 Days Training + 1 Day  Exam (35 hours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PECB CISO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PECB ISO 22301 (BCMS) Foundation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 days (16 hours)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PECB ISO 22301 (BCMS) Lead Auditor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PECB ISO 22301 (BCMS) Lead Implementer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PECB ISO/IEC 27001 (ISMS) Foundation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PECB ISO/IEC 27001 (ISMS) Lead Auditor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PECB ISO/IEC 27001 (ISMS) Lead Implementer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PECB ISO27001 (ISMS) Lead Auditor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RCC SOC Analyst &amp; Security Manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RCC Vulnerability Managers and Pen Testers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reverse Malware Engineering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scripting for Cybersecurity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOC Analyst and Security Manager​</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Study Techniques &amp; Exam Preparation​</t>
   </si>
   <si>
     <t xml:space="preserve">Vulnerability Assessment &amp; Penetration Testing (VAPT) Intermediate</t>
   </si>
   <si>
-    <t xml:space="preserve">Career Paths in Cybersecurity​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Careers in Cybersecurity: Entry​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Careers in Cybersecurity: Expert​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Careers in Cybersecurity: Specialist​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Advanced</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Careers in Cybersecurity: Management​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Study Techniques &amp; Exam Preparation​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SOC Analyst and Security Manager​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 Days​ (35 hours)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Incident Response, Threat Intelligence &amp; Digital Forensic Investigators </t>
-  </si>
-  <si>
     <t xml:space="preserve">Vulnerability Managers &amp; Pen Testers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CompTIA Tech+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 Days​ (24 hours)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CompTIA A+​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5 Days​ (40 hours)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CompTIA ​Server+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CompTIA Linux+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CompTIA Network+ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">CompTIA Security+</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CompTIA PenTest+​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CompTIA Cybersecurity Analyst (CySA+)​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ISC2 Certified in Cybersecurity Certification (CC)​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ISC2 Certified Information Systems Security Professional Certification (CISSP)​</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ISC2 Systems Security Certified Practitioner (SSCP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ISC2 Certified Secure Software Lifecycle Professional (CSSLP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ISC2 Governance, Risk and Compliance Certification (CGRC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EC-Council  Certified Ethical Hacker (CEH)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EC-Council Certified Chief Information Security Officer (CCISO)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PECB Certified Chief ​Information Security Officer (CISO)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 Days Training + 1 Day  Exam (35 hours)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PECB ISO/IEC 27001 (ISMS) Foundation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2 days (16 hours)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PECB ISO/IEC 27001 (ISMS) Lead Implementer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PECB ISO/IEC 27001 (ISMS) Lead Auditor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PECB ISO 22301 (BCMS) Foundation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PECB ISO 22301 (BCMS) Lead Implementer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PECB ISO 22301 (BCMS) Lead Auditor</t>
   </si>
 </sst>
 </file>
@@ -353,6 +401,31 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF4E95D9"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -593,13 +666,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
-  <sheetFormatPr defaultColWidth="34.15234375" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E65"/>
+  <sheetFormatPr defaultColWidth="34.15234375" defaultRowHeight="25.45" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="72.55"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="5" min="3" style="1" width="34.15"/>
   </cols>
   <sheetData>
-    <row r="1" s="3" customFormat="true" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -612,7 +686,7 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -625,7 +699,7 @@
       <c r="D2" s="5"/>
       <c r="E2" s="5"/>
     </row>
-    <row r="3" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -633,69 +707,69 @@
         <v>4</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D3" s="5"/>
       <c r="E3" s="5"/>
     </row>
-    <row r="4" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
     </row>
-    <row r="5" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
     </row>
-    <row r="6" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
     </row>
-    <row r="7" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
     </row>
-    <row r="8" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>14</v>
@@ -703,285 +777,285 @@
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
     </row>
-    <row r="9" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
         <v>15</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
-    <row r="10" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
-    <row r="11" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
         <v>18</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
     </row>
-    <row r="12" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
     </row>
-    <row r="13" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>22</v>
+    <row r="13" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>20</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
     </row>
-    <row r="14" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="s">
-        <v>23</v>
+    <row r="14" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>21</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
     </row>
-    <row r="15" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
     </row>
-    <row r="16" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
     </row>
-    <row r="17" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
     </row>
-    <row r="18" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
     </row>
-    <row r="19" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
     </row>
-    <row r="20" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
     </row>
-    <row r="21" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
     </row>
-    <row r="22" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
     </row>
-    <row r="23" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B23" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="4" t="s">
         <v>33</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>14</v>
       </c>
       <c r="D23" s="5"/>
       <c r="E23" s="5"/>
     </row>
-    <row r="24" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
     </row>
-    <row r="25" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
     </row>
-    <row r="26" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="D26" s="5"/>
       <c r="E26" s="5"/>
     </row>
-    <row r="27" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D27" s="5"/>
       <c r="E27" s="5"/>
     </row>
-    <row r="28" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D28" s="5"/>
       <c r="E28" s="5"/>
     </row>
-    <row r="29" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D29" s="5"/>
       <c r="E29" s="5"/>
     </row>
-    <row r="30" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>43</v>
@@ -989,12 +1063,12 @@
       <c r="D30" s="5"/>
       <c r="E30" s="5"/>
     </row>
-    <row r="31" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>43</v>
@@ -1002,12 +1076,12 @@
       <c r="D31" s="5"/>
       <c r="E31" s="5"/>
     </row>
-    <row r="32" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="s">
-        <v>46</v>
+    <row r="32" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
+        <v>45</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>43</v>
@@ -1015,46 +1089,46 @@
       <c r="D32" s="5"/>
       <c r="E32" s="5"/>
     </row>
-    <row r="33" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="D33" s="5"/>
       <c r="E33" s="5"/>
     </row>
-    <row r="34" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D34" s="5"/>
       <c r="E34" s="5"/>
     </row>
-    <row r="35" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="35" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>43</v>
       </c>
       <c r="D35" s="5"/>
       <c r="E35" s="5"/>
     </row>
-    <row r="36" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="36" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
         <v>50</v>
       </c>
@@ -1062,186 +1136,357 @@
         <v>4</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="D36" s="5"/>
       <c r="E36" s="5"/>
     </row>
-    <row r="37" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
         <v>51</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="D37" s="5"/>
       <c r="E37" s="5"/>
     </row>
-    <row r="38" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="38" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
         <v>52</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="D38" s="5"/>
       <c r="E38" s="5"/>
     </row>
-    <row r="39" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
         <v>53</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="D39" s="5"/>
       <c r="E39" s="5"/>
     </row>
-    <row r="40" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
         <v>54</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="D40" s="5"/>
       <c r="E40" s="5"/>
     </row>
-    <row r="41" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
         <v>55</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="D41" s="5"/>
       <c r="E41" s="5"/>
     </row>
-    <row r="42" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="42" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
         <v>56</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="D42" s="5"/>
       <c r="E42" s="5"/>
     </row>
-    <row r="43" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="43" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
         <v>57</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>58</v>
+        <v>11</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="D43" s="5"/>
       <c r="E43" s="5"/>
     </row>
-    <row r="44" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="6" t="s">
-        <v>59</v>
+    <row r="44" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
+        <v>58</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>60</v>
+        <v>16</v>
       </c>
       <c r="D44" s="5"/>
       <c r="E44" s="5"/>
     </row>
-    <row r="45" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>58</v>
+        <v>11</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="D45" s="5"/>
       <c r="E45" s="5"/>
     </row>
-    <row r="46" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>58</v>
+        <v>11</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="D46" s="5"/>
       <c r="E46" s="5"/>
     </row>
-    <row r="47" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="47" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="D47" s="5"/>
       <c r="E47" s="5"/>
     </row>
-    <row r="48" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="48" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>58</v>
+        <v>9</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>38</v>
       </c>
       <c r="D48" s="5"/>
       <c r="E48" s="5"/>
     </row>
-    <row r="49" s="3" customFormat="true" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="49" s="3" customFormat="true" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D49" s="5"/>
       <c r="E49" s="5"/>
     </row>
-    <row r="50" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3"/>
-      <c r="C50" s="5"/>
+    <row r="50" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>64</v>
+      </c>
       <c r="D50" s="5"/>
       <c r="E50" s="5"/>
+    </row>
+    <row r="51" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A57" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="25.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>41</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>